<commit_message>
docs: align design documents and agent docs
A cross-check of .agents against .docs found:
- Jira task descriptions cited .agents sections by number, and six of
  them pointed at the wrong section after the rewrite; cite them by
  section name so reordering cannot break them again.
- The data dictionary did not record ON DELETE behaviour; column Khóa
  now marks the 21 CASCADE and 2 SET NULL foreign keys of the backend
  migrations, and coding_rule.md points there instead of keeping an
  incomplete list.
- API design 1.8 states that the general rate limit is per IP when
  anonymous, as the backend already does.
- .agents gains the access rules, Admin permissions, date format and
  RM-14 details that only the API design had, and no longer says every
  delete returns null data (BLOG-09 returns the like count).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.docs/ANGI_Jira_Plan_Ver1.2.xlsx
+++ b/.docs/ANGI_Jira_Plan_Ver1.2.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprints" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workload" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sprints" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Team" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Epics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gantt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Workload" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$O$212</definedName>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>8.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Mỗi dev chạy được DB local bằng 1 lệnh; tạo 2 DB role riêng cho backend (schema core) và reco (schema recommendation) như project_architecture.md mục 6. Viết hướng dẫn chạy vào README. Tạo .env.example (backend, reco, frontend) liệt kê đủ key ngoài và tự đăng ký key dùng chung cho dev: Google OAuth ClientId, Brevo ApiKey + sender, Cloudinary (CloudName, ApiKey, ApiSecret), Mapbox secret token (backend) và public token pk.* (frontend), key LLM (reco), X-Api-Key backend ↔ reco. Gửi key cho team qua kênh riêng, không commit (local dùng user-secrets / .env).</t>
+          <t>Mỗi dev chạy được DB local bằng 1 lệnh; tạo 2 DB role riêng cho backend (schema core) và reco (schema recommendation) như project_architecture.md, mục Database. Viết hướng dẫn chạy vào README. Tạo .env.example (backend, reco, frontend) liệt kê đủ key ngoài và tự đăng ký key dùng chung cho dev: Google OAuth ClientId, Brevo ApiKey + sender, Cloudinary (CloudName, ApiKey, ApiSecret), Mapbox secret token (backend) và public token pk.* (frontend), key LLM (reco), X-Api-Key backend ↔ reco. Gửi key cho team qua kênh riêng, không commit (local dùng user-secrets / .env).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md mục 2). Dùng cho MEDIA-01 và bảng media_files.</t>
+          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md, mục Integrations). Dùng cho MEDIA-01 và bảng media_files.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md mục 2). Dùng cho F-01, F-02, F-05.</t>
+          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md, mục Integrations). Dùng cho F-01, F-02, F-05.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Map toàn bộ bảng schema core theo ANGI_Data_Dictionary_Ver1.2 vào ANGIContext (IEntityTypeConfiguration mỗi bảng), BaseEntity + ISoftDelete, enum lưu đúng giá trị chữ thường như sheet Enum của ANGI_API_Design_Ver1.8. Initial migration gồm cả CHECK, citext và trigger outbox (migrationBuilder.Sql). Từ đây schema core chỉ đổi qua EF migration (commit_guide.md mục 10). | Làm sau: Docker Compose môi trường dev: PostgreSQL 16 + pgvector.</t>
+          <t>Map toàn bộ bảng schema core theo ANGI_Data_Dictionary_Ver1.2 vào ANGIContext (IEntityTypeConfiguration mỗi bảng), BaseEntity + ISoftDelete, enum lưu đúng giá trị chữ thường như sheet Enum của ANGI_API_Design_Ver1.8. Initial migration gồm cả CHECK, citext và trigger outbox (migrationBuilder.Sql). Từ đây schema core chỉ đổi qua EF migration (commit_guide.md, mục Migrations). | Làm sau: Docker Compose môi trường dev: PostgreSQL 16 + pgvector.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mọi response bọc trong ApiResponse&lt;T&gt; (success, message, errorCode, data, errors) theo coding_rule.md mục 5. Middleware map exception sang status + errorCode theo coding_rule.md mục 7 và sheet Mã lỗi của ANGI_API_Design_Ver1.8; 401, 403, 429 và lỗi model binding cũng trả ApiResponse. JWT, CORS, rate limit theo project_architecture.md mục 4–5.</t>
+          <t>Mọi response bọc trong ApiResponse&lt;T&gt; (success, message, errorCode, data, errors) theo coding_rule.md, mục Responses. Middleware map exception sang status + errorCode theo coding_rule.md, mục Errors và sheet Mã lỗi của ANGI_API_Design_Ver1.8; 401, 403, 429 và lỗi model binding cũng trả ApiResponse. JWT, CORS, rate limit theo project_architecture.md, mục Request pipeline và API conventions.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Typed HttpClient gọi RECO-03, RECO-05, RECO-06, RECO-09 với X-Api-Key; timeout 800 ms và fallback xếp theo rating quán (project_architecture.md mục 2). | Làm sau: Khung FastAPI reco service: kết nối schema recommendation, migration, X-Api-Key, /health.</t>
+          <t>Typed HttpClient gọi RECO-03, RECO-05, RECO-06, RECO-09 với X-Api-Key; timeout 800 ms và fallback xếp theo rating quán (project_architecture.md, mục Integrations). | Làm sau: Khung FastAPI reco service: kết nối schema recommendation, migration, X-Api-Key, /health.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>8.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
 Endpoint cần làm:
 - HOME-01 GET /api/v1/home
 - IMP-01 POST /api/v1/impressions
-Ghi chú: Món gợi ý lấy qua IRecommendationService (RECO-05). Reco lỗi hoặc quá 800 ms thì xếp theo rating quán (project_architecture.md mục 2). Code trước với bản mock của IRecommendationService (trả lại candidate_dish_ids đúng thứ tự gửi, requestId = null, giống fallback) để không phải chờ RECO-05; reco xong chỉ đổi đăng ký DI. Ứng viên gửi RECO-05 sắp sẵn theo rating trung bình của quán giảm dần, rồi like_count của món giảm dần (reco giữ thứ tự này cho món bằng điểm). Lọc xong còn quá 2000 món thì chỉ gửi 2000 món đầu (RECO-05 nhận tối đa 2000).
+Ghi chú: Món gợi ý lấy qua IRecommendationService (RECO-05). Reco lỗi hoặc quá 800 ms thì xếp theo rating quán (project_architecture.md, mục Integrations). Code trước với bản mock của IRecommendationService (trả lại candidate_dish_ids đúng thứ tự gửi, requestId = null, giống fallback) để không phải chờ RECO-05; reco xong chỉ đổi đăng ký DI. Ứng viên gửi RECO-05 sắp sẵn theo rating trung bình của quán giảm dần, rồi like_count của món giảm dần (reco giữ thứ tự này cho món bằng điểm). Lọc xong còn quá 2000 món thì chỉ gửi 2000 món đầu (RECO-05 nhận tối đa 2000).
 Tài liệu: ANGI_Use_Case_Basic_Descriptions_Ver1.0 (use case), ANGI_API_Design_Ver1.8 (sheet Backend API, Chi tiết Request-Response, Mã lỗi), ANGI_Data_Dictionary_Ver1.2 (bảng), coding_rule.md.
 DoD: Endpoint trả đúng request/response và mã lỗi như ANGI_API_Design_Ver1.8; code theo coding_rule.md; unit test tối thiểu 2 method; hiện trên Scalar; PR được Dũng review. | Làm sau: Reco P1: Cold start (Pooled Wilson) + Content-based, RECO-05 /recommendations, RECO-06 /impressions.</t>
         </is>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>BackgroundService đọc outbox_messages, gửi kèm Idempotency-Key, thử lại theo backoff, chuyển dead khi lỗi 4xx hoặc quá số lần thử. Chi tiết luồng: project_architecture.md mục 7. | Làm sau: Reco P1: Sinh dish vector (RECO-01 upsert, RECO-02 deactivate), [BE] F-50 Manage Restaurant Menu.</t>
+          <t>BackgroundService đọc outbox_messages, gửi kèm Idempotency-Key, thử lại theo backoff, chuyển dead khi lỗi 4xx hoặc quá số lần thử. Chi tiết luồng: project_architecture.md, mục Outbox. | Làm sau: Reco P1: Sinh dish vector (RECO-01 upsert, RECO-02 deactivate), [BE] F-50 Manage Restaurant Menu.</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -6534,7 +6534,7 @@
           <t>[CRITICAL PATH] Task này nằm trên đường găng: dự phòng tối đa 1 ngày. Phải xong đúng Due Date 20/10/2026; trễ 1 ngày thì mốc "Software Package Version 1" (25/10/2026) bị trễ theo.
 Ảnh hưởng trực tiếp tới: Code freeze + tích hợp Iteration 1: merge PR vào dev, chạy toàn hệ thống.
 Gặp vướng thì báo ngay trong ngày cho Dũng (PM), không đợi họp.
-Interface IRouteService ở Application/Common/Interfaces/Services, MapboxRouteService ở Infrastructure/Services (typed HttpClient gọi Mapbox Directions API, 1 lần cho cả ngày, tối đa 25 điểm). Cache IMemoryCache 24 giờ theo profile + tọa độ (điểm xuất phát làm tròn khoảng 100 m); timeout 3 giây, lỗi thì ước lượng đường chim bay × 1,3 và trả isEstimated = true. Tạo tài khoản Mapbox, secret token để ở biến môi trường (Mapbox__AccessToken), public token cho FE. Chi tiết project_architecture.md mục 2 (Map / routing). Dùng cho RM-14 ở F-21 (Iteration 2).</t>
+Interface IRouteService ở Application/Common/Interfaces/Services, MapboxRouteService ở Infrastructure/Services (typed HttpClient gọi Mapbox Directions API, 1 lần cho cả ngày, tối đa 25 điểm). Cache IMemoryCache 24 giờ theo profile + tọa độ (điểm xuất phát làm tròn khoảng 100 m); timeout 3 giây, lỗi thì ước lượng đường chim bay × 1,3 và trả isEstimated = true. Tạo tài khoản Mapbox, secret token để ở biến môi trường (Mapbox__AccessToken), public token cho FE. Chi tiết project_architecture.md, mục Integrations (Mapbox Directions). Dùng cho RM-14 ở F-21 (Iteration 2).</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="M89" s="2" t="inlineStr"/>
       <c r="N89" s="2" t="n">
-        <v>9.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -13223,7 +13223,7 @@
       </c>
       <c r="M160" s="2" t="inlineStr"/>
       <c r="N160" s="2" t="n">
-        <v>8.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
@@ -17660,7 +17660,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G2" s="6" t="n"/>
       <c r="L2" s="7" t="n"/>
@@ -18701,7 +18701,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>8.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
@@ -22139,7 +22139,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>9.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L89" s="7" t="n"/>
       <c r="M89" s="7" t="n"/>
@@ -25781,7 +25781,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>8.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
@@ -28719,6 +28719,7 @@
         <v>99</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: align design documents and agent docs (#17)
Cite .agents sections by name in the Jira plan, record ON DELETE
behaviour in the data dictionary, state the per-IP anonymous rate limit
in the API design, and bring the access, date and RM-14 rules into the
agent docs.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.docs/ANGI_Jira_Plan_Ver1.2.xlsx
+++ b/.docs/ANGI_Jira_Plan_Ver1.2.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprints" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workload" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sprints" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Team" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Epics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gantt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Workload" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$O$212</definedName>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>8.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Mỗi dev chạy được DB local bằng 1 lệnh; tạo 2 DB role riêng cho backend (schema core) và reco (schema recommendation) như project_architecture.md mục 6. Viết hướng dẫn chạy vào README. Tạo .env.example (backend, reco, frontend) liệt kê đủ key ngoài và tự đăng ký key dùng chung cho dev: Google OAuth ClientId, Brevo ApiKey + sender, Cloudinary (CloudName, ApiKey, ApiSecret), Mapbox secret token (backend) và public token pk.* (frontend), key LLM (reco), X-Api-Key backend ↔ reco. Gửi key cho team qua kênh riêng, không commit (local dùng user-secrets / .env).</t>
+          <t>Mỗi dev chạy được DB local bằng 1 lệnh; tạo 2 DB role riêng cho backend (schema core) và reco (schema recommendation) như project_architecture.md, mục Database. Viết hướng dẫn chạy vào README. Tạo .env.example (backend, reco, frontend) liệt kê đủ key ngoài và tự đăng ký key dùng chung cho dev: Google OAuth ClientId, Brevo ApiKey + sender, Cloudinary (CloudName, ApiKey, ApiSecret), Mapbox secret token (backend) và public token pk.* (frontend), key LLM (reco), X-Api-Key backend ↔ reco. Gửi key cho team qua kênh riêng, không commit (local dùng user-secrets / .env).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md mục 2). Dùng cho MEDIA-01 và bảng media_files.</t>
+          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md, mục Integrations). Dùng cho MEDIA-01 và bảng media_files.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md mục 2). Dùng cho F-01, F-02, F-05.</t>
+          <t>Interface ở Application/Common/Interfaces/Services, implementation ở Infrastructure/Services (project_architecture.md, mục Integrations). Dùng cho F-01, F-02, F-05.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Map toàn bộ bảng schema core theo ANGI_Data_Dictionary_Ver1.2 vào ANGIContext (IEntityTypeConfiguration mỗi bảng), BaseEntity + ISoftDelete, enum lưu đúng giá trị chữ thường như sheet Enum của ANGI_API_Design_Ver1.8. Initial migration gồm cả CHECK, citext và trigger outbox (migrationBuilder.Sql). Từ đây schema core chỉ đổi qua EF migration (commit_guide.md mục 10). | Làm sau: Docker Compose môi trường dev: PostgreSQL 16 + pgvector.</t>
+          <t>Map toàn bộ bảng schema core theo ANGI_Data_Dictionary_Ver1.2 vào ANGIContext (IEntityTypeConfiguration mỗi bảng), BaseEntity + ISoftDelete, enum lưu đúng giá trị chữ thường như sheet Enum của ANGI_API_Design_Ver1.8. Initial migration gồm cả CHECK, citext và trigger outbox (migrationBuilder.Sql). Từ đây schema core chỉ đổi qua EF migration (commit_guide.md, mục Migrations). | Làm sau: Docker Compose môi trường dev: PostgreSQL 16 + pgvector.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mọi response bọc trong ApiResponse&lt;T&gt; (success, message, errorCode, data, errors) theo coding_rule.md mục 5. Middleware map exception sang status + errorCode theo coding_rule.md mục 7 và sheet Mã lỗi của ANGI_API_Design_Ver1.8; 401, 403, 429 và lỗi model binding cũng trả ApiResponse. JWT, CORS, rate limit theo project_architecture.md mục 4–5.</t>
+          <t>Mọi response bọc trong ApiResponse&lt;T&gt; (success, message, errorCode, data, errors) theo coding_rule.md, mục Responses. Middleware map exception sang status + errorCode theo coding_rule.md, mục Errors và sheet Mã lỗi của ANGI_API_Design_Ver1.8; 401, 403, 429 và lỗi model binding cũng trả ApiResponse. JWT, CORS, rate limit theo project_architecture.md, mục Request pipeline và API conventions.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Typed HttpClient gọi RECO-03, RECO-05, RECO-06, RECO-09 với X-Api-Key; timeout 800 ms và fallback xếp theo rating quán (project_architecture.md mục 2). | Làm sau: Khung FastAPI reco service: kết nối schema recommendation, migration, X-Api-Key, /health.</t>
+          <t>Typed HttpClient gọi RECO-03, RECO-05, RECO-06, RECO-09 với X-Api-Key; timeout 800 ms và fallback xếp theo rating quán (project_architecture.md, mục Integrations). | Làm sau: Khung FastAPI reco service: kết nối schema recommendation, migration, X-Api-Key, /health.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>8.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
 Endpoint cần làm:
 - HOME-01 GET /api/v1/home
 - IMP-01 POST /api/v1/impressions
-Ghi chú: Món gợi ý lấy qua IRecommendationService (RECO-05). Reco lỗi hoặc quá 800 ms thì xếp theo rating quán (project_architecture.md mục 2). Code trước với bản mock của IRecommendationService (trả lại candidate_dish_ids đúng thứ tự gửi, requestId = null, giống fallback) để không phải chờ RECO-05; reco xong chỉ đổi đăng ký DI. Ứng viên gửi RECO-05 sắp sẵn theo rating trung bình của quán giảm dần, rồi like_count của món giảm dần (reco giữ thứ tự này cho món bằng điểm). Lọc xong còn quá 2000 món thì chỉ gửi 2000 món đầu (RECO-05 nhận tối đa 2000).
+Ghi chú: Món gợi ý lấy qua IRecommendationService (RECO-05). Reco lỗi hoặc quá 800 ms thì xếp theo rating quán (project_architecture.md, mục Integrations). Code trước với bản mock của IRecommendationService (trả lại candidate_dish_ids đúng thứ tự gửi, requestId = null, giống fallback) để không phải chờ RECO-05; reco xong chỉ đổi đăng ký DI. Ứng viên gửi RECO-05 sắp sẵn theo rating trung bình của quán giảm dần, rồi like_count của món giảm dần (reco giữ thứ tự này cho món bằng điểm). Lọc xong còn quá 2000 món thì chỉ gửi 2000 món đầu (RECO-05 nhận tối đa 2000).
 Tài liệu: ANGI_Use_Case_Basic_Descriptions_Ver1.0 (use case), ANGI_API_Design_Ver1.8 (sheet Backend API, Chi tiết Request-Response, Mã lỗi), ANGI_Data_Dictionary_Ver1.2 (bảng), coding_rule.md.
 DoD: Endpoint trả đúng request/response và mã lỗi như ANGI_API_Design_Ver1.8; code theo coding_rule.md; unit test tối thiểu 2 method; hiện trên Scalar; PR được Dũng review. | Làm sau: Reco P1: Cold start (Pooled Wilson) + Content-based, RECO-05 /recommendations, RECO-06 /impressions.</t>
         </is>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>BackgroundService đọc outbox_messages, gửi kèm Idempotency-Key, thử lại theo backoff, chuyển dead khi lỗi 4xx hoặc quá số lần thử. Chi tiết luồng: project_architecture.md mục 7. | Làm sau: Reco P1: Sinh dish vector (RECO-01 upsert, RECO-02 deactivate), [BE] F-50 Manage Restaurant Menu.</t>
+          <t>BackgroundService đọc outbox_messages, gửi kèm Idempotency-Key, thử lại theo backoff, chuyển dead khi lỗi 4xx hoặc quá số lần thử. Chi tiết luồng: project_architecture.md, mục Outbox. | Làm sau: Reco P1: Sinh dish vector (RECO-01 upsert, RECO-02 deactivate), [BE] F-50 Manage Restaurant Menu.</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -6534,7 +6534,7 @@
           <t>[CRITICAL PATH] Task này nằm trên đường găng: dự phòng tối đa 1 ngày. Phải xong đúng Due Date 20/10/2026; trễ 1 ngày thì mốc "Software Package Version 1" (25/10/2026) bị trễ theo.
 Ảnh hưởng trực tiếp tới: Code freeze + tích hợp Iteration 1: merge PR vào dev, chạy toàn hệ thống.
 Gặp vướng thì báo ngay trong ngày cho Dũng (PM), không đợi họp.
-Interface IRouteService ở Application/Common/Interfaces/Services, MapboxRouteService ở Infrastructure/Services (typed HttpClient gọi Mapbox Directions API, 1 lần cho cả ngày, tối đa 25 điểm). Cache IMemoryCache 24 giờ theo profile + tọa độ (điểm xuất phát làm tròn khoảng 100 m); timeout 3 giây, lỗi thì ước lượng đường chim bay × 1,3 và trả isEstimated = true. Tạo tài khoản Mapbox, secret token để ở biến môi trường (Mapbox__AccessToken), public token cho FE. Chi tiết project_architecture.md mục 2 (Map / routing). Dùng cho RM-14 ở F-21 (Iteration 2).</t>
+Interface IRouteService ở Application/Common/Interfaces/Services, MapboxRouteService ở Infrastructure/Services (typed HttpClient gọi Mapbox Directions API, 1 lần cho cả ngày, tối đa 25 điểm). Cache IMemoryCache 24 giờ theo profile + tọa độ (điểm xuất phát làm tròn khoảng 100 m); timeout 3 giây, lỗi thì ước lượng đường chim bay × 1,3 và trả isEstimated = true. Tạo tài khoản Mapbox, secret token để ở biến môi trường (Mapbox__AccessToken), public token cho FE. Chi tiết project_architecture.md, mục Integrations (Mapbox Directions). Dùng cho RM-14 ở F-21 (Iteration 2).</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="M89" s="2" t="inlineStr"/>
       <c r="N89" s="2" t="n">
-        <v>9.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -13223,7 +13223,7 @@
       </c>
       <c r="M160" s="2" t="inlineStr"/>
       <c r="N160" s="2" t="n">
-        <v>8.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
@@ -17660,7 +17660,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G2" s="6" t="n"/>
       <c r="L2" s="7" t="n"/>
@@ -18701,7 +18701,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>8.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
@@ -22139,7 +22139,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>9.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L89" s="7" t="n"/>
       <c r="M89" s="7" t="n"/>
@@ -25781,7 +25781,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>8.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
@@ -28719,6 +28719,7 @@
         <v>99</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(agent): define roadmap conversation contracts
Document AGENT-01..04, integer identities, schema invariants and the
acceptance cases alongside the API and data dictionary. Preserve the
latest dev clarifications while adding the Agent module.

Refs: ANGI-231
</commit_message>
<xml_diff>
--- a/.docs/ANGI_Jira_Plan_Ver1.2.xlsx
+++ b/.docs/ANGI_Jira_Plan_Ver1.2.xlsx
@@ -15,9 +15,9 @@
     <sheet name="Workload" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$O$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$O$213</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:Z7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -870,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:Z14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1359,7 +1359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O212"/>
+  <dimension ref="A1:O213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1515,7 +1515,7 @@
           <t>ANGI-14</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="2"/>
       <c r="N2" s="2" t="n">
         <v>8.300000000000001</v>
       </c>
@@ -1584,7 +1584,7 @@
           <t>ANGI-15</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2"/>
       <c r="N3" s="2" t="n">
         <v>69</v>
       </c>
@@ -1653,7 +1653,7 @@
           <t>ANGI-16</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2"/>
       <c r="N4" s="2" t="n">
         <v>8.5</v>
       </c>
@@ -1722,7 +1722,7 @@
           <t>ANGI-17</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="M5" s="2"/>
       <c r="N5" s="2" t="n">
         <v>11.5</v>
       </c>
@@ -1791,7 +1791,7 @@
           <t>ANGI-18</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="M6" s="2"/>
       <c r="N6" s="2" t="n">
         <v>10.8</v>
       </c>
@@ -1860,7 +1860,7 @@
           <t>ANGI-19</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2"/>
       <c r="N7" s="2" t="n">
         <v>8.1</v>
       </c>
@@ -1929,7 +1929,7 @@
           <t>ANGI-20</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="M8" s="2"/>
       <c r="N8" s="2" t="n">
         <v>8.1</v>
       </c>
@@ -1998,7 +1998,7 @@
           <t>ANGI-21</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2"/>
       <c r="N9" s="2" t="n">
         <v>8.5</v>
       </c>
@@ -2067,7 +2067,7 @@
           <t>ANGI-22</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="M10" s="2"/>
       <c r="N10" s="2" t="n">
         <v>66</v>
       </c>
@@ -2136,7 +2136,7 @@
           <t>ANGI-23</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="M11" s="2"/>
       <c r="N11" s="2" t="n">
         <v>6.4</v>
       </c>
@@ -2205,7 +2205,7 @@
           <t>ANGI-24</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2"/>
       <c r="N12" s="2" t="n">
         <v>65.8</v>
       </c>
@@ -2274,7 +2274,7 @@
           <t>ANGI-25</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="M13" s="2"/>
       <c r="N13" s="2" t="n">
         <v>63</v>
       </c>
@@ -2343,7 +2343,7 @@
           <t>ANGI-26</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2"/>
       <c r="N14" s="2" t="n">
         <v>7.4</v>
       </c>
@@ -2412,7 +2412,7 @@
           <t>ANGI-27</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2"/>
       <c r="N15" s="2" t="n">
         <v>63</v>
       </c>
@@ -2481,7 +2481,7 @@
           <t>ANGI-28</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="M16" s="2"/>
       <c r="N16" s="2" t="n">
         <v>3.1</v>
       </c>
@@ -2555,7 +2555,7 @@
           <t>ANGI-29</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2"/>
       <c r="N17" s="2" t="n">
         <v>7.3</v>
       </c>
@@ -2628,7 +2628,7 @@
           <t>ANGI-30</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2"/>
       <c r="N18" s="2" t="n">
         <v>9.4</v>
       </c>
@@ -2701,7 +2701,7 @@
           <t>ANGI-31</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="M19" s="2"/>
       <c r="N19" s="2" t="n">
         <v>7.2</v>
       </c>
@@ -2770,7 +2770,7 @@
           <t>ANGI-32</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2"/>
       <c r="N20" s="2" t="n">
         <v>5.7</v>
       </c>
@@ -2846,7 +2846,7 @@
           <t>ANGI-33</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2"/>
       <c r="N21" s="2" t="n">
         <v>6.1</v>
       </c>
@@ -2921,7 +2921,7 @@
           <t>ANGI-34</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="M22" s="2"/>
       <c r="N22" s="2" t="n">
         <v>8.699999999999999</v>
       </c>
@@ -2996,7 +2996,7 @@
           <t>ANGI-35</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2"/>
       <c r="N23" s="2" t="n">
         <v>6.7</v>
       </c>
@@ -3070,7 +3070,7 @@
           <t>ANGI-36</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2"/>
       <c r="N24" s="2" t="n">
         <v>8.9</v>
       </c>
@@ -3139,7 +3139,7 @@
           <t>ANGI-37</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2"/>
       <c r="N25" s="2" t="n">
         <v>2.4</v>
       </c>
@@ -3214,7 +3214,7 @@
           <t>ANGI-38</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2"/>
       <c r="N26" s="2" t="n">
         <v>6.1</v>
       </c>
@@ -3288,7 +3288,7 @@
           <t>ANGI-39</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2"/>
       <c r="N27" s="2" t="n">
         <v>6</v>
       </c>
@@ -3362,7 +3362,7 @@
           <t>ANGI-40</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="M28" s="2"/>
       <c r="N28" s="2" t="n">
         <v>5.8</v>
       </c>
@@ -3435,7 +3435,7 @@
           <t>ANGI-41</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2"/>
       <c r="N29" s="2" t="n">
         <v>7.8</v>
       </c>
@@ -3509,7 +3509,7 @@
           <t>ANGI-42</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2"/>
       <c r="N30" s="2" t="n">
         <v>5.4</v>
       </c>
@@ -3583,7 +3583,7 @@
           <t>ANGI-43</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr"/>
+      <c r="M31" s="2"/>
       <c r="N31" s="2" t="n">
         <v>7.8</v>
       </c>
@@ -3652,7 +3652,7 @@
           <t>ANGI-44</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr"/>
+      <c r="M32" s="2"/>
       <c r="N32" s="2" t="n">
         <v>2.4</v>
       </c>
@@ -3721,7 +3721,7 @@
           <t>ANGI-45</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
+      <c r="M33" s="2"/>
       <c r="N33" s="2" t="n">
         <v>60</v>
       </c>
@@ -3796,7 +3796,7 @@
           <t>ANGI-46</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr"/>
+      <c r="M34" s="2"/>
       <c r="N34" s="2" t="n">
         <v>7.1</v>
       </c>
@@ -3869,7 +3869,7 @@
           <t>ANGI-47</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
+      <c r="M35" s="2"/>
       <c r="N35" s="2" t="n">
         <v>5.3</v>
       </c>
@@ -3942,7 +3942,7 @@
           <t>ANGI-48</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
+      <c r="M36" s="2"/>
       <c r="N36" s="2" t="n">
         <v>7</v>
       </c>
@@ -4015,7 +4015,7 @@
           <t>ANGI-49</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr"/>
+      <c r="M37" s="2"/>
       <c r="N37" s="2" t="n">
         <v>5</v>
       </c>
@@ -4167,7 +4167,7 @@
           <t>ANGI-51</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
+      <c r="M39" s="2"/>
       <c r="N39" s="2" t="n">
         <v>6.5</v>
       </c>
@@ -4240,7 +4240,7 @@
           <t>ANGI-52</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr"/>
+      <c r="M40" s="2"/>
       <c r="N40" s="2" t="n">
         <v>4.8</v>
       </c>
@@ -4322,7 +4322,7 @@
           <t>ANGI-53</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr"/>
+      <c r="M41" s="2"/>
       <c r="N41" s="2" t="n">
         <v>4.3</v>
       </c>
@@ -4395,7 +4395,7 @@
           <t>ANGI-54</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr"/>
+      <c r="M42" s="2"/>
       <c r="N42" s="2" t="n">
         <v>6.1</v>
       </c>
@@ -4468,7 +4468,7 @@
           <t>ANGI-55</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr"/>
+      <c r="M43" s="2"/>
       <c r="N43" s="2" t="n">
         <v>6.6</v>
       </c>
@@ -4541,7 +4541,7 @@
           <t>ANGI-56</t>
         </is>
       </c>
-      <c r="M44" s="2" t="inlineStr"/>
+      <c r="M44" s="2"/>
       <c r="N44" s="2" t="n">
         <v>4.2</v>
       </c>
@@ -4693,7 +4693,7 @@
           <t>ANGI-58</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr"/>
+      <c r="M46" s="2"/>
       <c r="N46" s="2" t="n">
         <v>3.8</v>
       </c>
@@ -4767,7 +4767,7 @@
           <t>ANGI-59</t>
         </is>
       </c>
-      <c r="M47" s="2" t="inlineStr"/>
+      <c r="M47" s="2"/>
       <c r="N47" s="2" t="n">
         <v>5.8</v>
       </c>
@@ -4840,7 +4840,7 @@
           <t>ANGI-60</t>
         </is>
       </c>
-      <c r="M48" s="2" t="inlineStr"/>
+      <c r="M48" s="2"/>
       <c r="N48" s="2" t="n">
         <v>3.7</v>
       </c>
@@ -4914,7 +4914,7 @@
           <t>ANGI-61</t>
         </is>
       </c>
-      <c r="M49" s="2" t="inlineStr"/>
+      <c r="M49" s="2"/>
       <c r="N49" s="2" t="n">
         <v>5.5</v>
       </c>
@@ -4988,7 +4988,7 @@
           <t>ANGI-62</t>
         </is>
       </c>
-      <c r="M50" s="2" t="inlineStr"/>
+      <c r="M50" s="2"/>
       <c r="N50" s="2" t="n">
         <v>3.2</v>
       </c>
@@ -5061,7 +5061,7 @@
           <t>ANGI-63</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr"/>
+      <c r="M51" s="2"/>
       <c r="N51" s="2" t="n">
         <v>5.2</v>
       </c>
@@ -5135,7 +5135,7 @@
           <t>ANGI-64</t>
         </is>
       </c>
-      <c r="M52" s="2" t="inlineStr"/>
+      <c r="M52" s="2"/>
       <c r="N52" s="2" t="n">
         <v>3.4</v>
       </c>
@@ -5208,7 +5208,7 @@
           <t>ANGI-65</t>
         </is>
       </c>
-      <c r="M53" s="2" t="inlineStr"/>
+      <c r="M53" s="2"/>
       <c r="N53" s="2" t="n">
         <v>5.1</v>
       </c>
@@ -5282,7 +5282,7 @@
           <t>ANGI-66</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr"/>
+      <c r="M54" s="2"/>
       <c r="N54" s="2" t="n">
         <v>2.8</v>
       </c>
@@ -5356,7 +5356,7 @@
           <t>ANGI-67</t>
         </is>
       </c>
-      <c r="M55" s="2" t="inlineStr"/>
+      <c r="M55" s="2"/>
       <c r="N55" s="2" t="n">
         <v>4.9</v>
       </c>
@@ -5429,7 +5429,7 @@
           <t>ANGI-68</t>
         </is>
       </c>
-      <c r="M56" s="2" t="inlineStr"/>
+      <c r="M56" s="2"/>
       <c r="N56" s="2" t="n">
         <v>4.4</v>
       </c>
@@ -5587,7 +5587,7 @@
           <t>ANGI-70</t>
         </is>
       </c>
-      <c r="M58" s="2" t="inlineStr"/>
+      <c r="M58" s="2"/>
       <c r="N58" s="2" t="n">
         <v>2.3</v>
       </c>
@@ -5662,7 +5662,7 @@
           <t>ANGI-71</t>
         </is>
       </c>
-      <c r="M59" s="2" t="inlineStr"/>
+      <c r="M59" s="2"/>
       <c r="N59" s="2" t="n">
         <v>2</v>
       </c>
@@ -5821,7 +5821,7 @@
           <t>ANGI-73</t>
         </is>
       </c>
-      <c r="M61" s="2" t="inlineStr"/>
+      <c r="M61" s="2"/>
       <c r="N61" s="2" t="n">
         <v>3.9</v>
       </c>
@@ -5896,7 +5896,7 @@
           <t>ANGI-74</t>
         </is>
       </c>
-      <c r="M62" s="2" t="inlineStr"/>
+      <c r="M62" s="2"/>
       <c r="N62" s="2" t="n">
         <v>3.6</v>
       </c>
@@ -5970,7 +5970,7 @@
           <t>ANGI-75</t>
         </is>
       </c>
-      <c r="M63" s="2" t="inlineStr"/>
+      <c r="M63" s="2"/>
       <c r="N63" s="2" t="n">
         <v>1.7</v>
       </c>
@@ -6120,7 +6120,7 @@
           <t>ANGI-77</t>
         </is>
       </c>
-      <c r="M65" s="2" t="inlineStr"/>
+      <c r="M65" s="2"/>
       <c r="N65" s="2" t="n">
         <v>3</v>
       </c>
@@ -6276,7 +6276,7 @@
           <t>ANGI-79</t>
         </is>
       </c>
-      <c r="M67" s="2" t="inlineStr"/>
+      <c r="M67" s="2"/>
       <c r="N67" s="2" t="n">
         <v>2.9</v>
       </c>
@@ -6357,7 +6357,7 @@
           <t>ANGI-80</t>
         </is>
       </c>
-      <c r="M68" s="2" t="inlineStr"/>
+      <c r="M68" s="2"/>
       <c r="N68" s="2" t="n">
         <v>1.8</v>
       </c>
@@ -6430,7 +6430,7 @@
           <t>ANGI-81</t>
         </is>
       </c>
-      <c r="M69" s="2" t="inlineStr"/>
+      <c r="M69" s="2"/>
       <c r="N69" s="2" t="n">
         <v>2.6</v>
       </c>
@@ -6503,7 +6503,7 @@
           <t>ANGI-82</t>
         </is>
       </c>
-      <c r="M70" s="2" t="inlineStr"/>
+      <c r="M70" s="2"/>
       <c r="N70" s="2" t="n">
         <v>2.3</v>
       </c>
@@ -6652,7 +6652,7 @@
           <t>ANGI-83</t>
         </is>
       </c>
-      <c r="M72" s="2" t="inlineStr"/>
+      <c r="M72" s="2"/>
       <c r="N72" s="2" t="n">
         <v>1.6</v>
       </c>
@@ -6721,7 +6721,7 @@
           <t>ANGI-84</t>
         </is>
       </c>
-      <c r="M73" s="2" t="inlineStr"/>
+      <c r="M73" s="2"/>
       <c r="N73" s="2" t="n">
         <v>4</v>
       </c>
@@ -6955,7 +6955,7 @@
           <t>ANGI-87</t>
         </is>
       </c>
-      <c r="M76" s="2" t="inlineStr"/>
+      <c r="M76" s="2"/>
       <c r="N76" s="2" t="n">
         <v>54</v>
       </c>
@@ -7634,7 +7634,7 @@
           <t>ANGI-96</t>
         </is>
       </c>
-      <c r="M85" s="2" t="inlineStr"/>
+      <c r="M85" s="2"/>
       <c r="N85" s="2" t="n">
         <v>8.5</v>
       </c>
@@ -7703,7 +7703,7 @@
           <t>ANGI-97</t>
         </is>
       </c>
-      <c r="M86" s="2" t="inlineStr"/>
+      <c r="M86" s="2"/>
       <c r="N86" s="2" t="n">
         <v>50</v>
       </c>
@@ -7853,7 +7853,7 @@
           <t>ANGI-99</t>
         </is>
       </c>
-      <c r="M88" s="2" t="inlineStr"/>
+      <c r="M88" s="2"/>
       <c r="N88" s="2" t="n">
         <v>7.5</v>
       </c>
@@ -7927,7 +7927,7 @@
           <t>ANGI-100</t>
         </is>
       </c>
-      <c r="M89" s="2" t="inlineStr"/>
+      <c r="M89" s="2"/>
       <c r="N89" s="2" t="n">
         <v>9.300000000000001</v>
       </c>
@@ -8000,7 +8000,7 @@
           <t>ANGI-101</t>
         </is>
       </c>
-      <c r="M90" s="2" t="inlineStr"/>
+      <c r="M90" s="2"/>
       <c r="N90" s="2" t="n">
         <v>7.3</v>
       </c>
@@ -8069,7 +8069,7 @@
           <t>ANGI-102</t>
         </is>
       </c>
-      <c r="M91" s="2" t="inlineStr"/>
+      <c r="M91" s="2"/>
       <c r="N91" s="2" t="n">
         <v>6.3</v>
       </c>
@@ -8142,7 +8142,7 @@
           <t>ANGI-103</t>
         </is>
       </c>
-      <c r="M92" s="2" t="inlineStr"/>
+      <c r="M92" s="2"/>
       <c r="N92" s="2" t="n">
         <v>8.9</v>
       </c>
@@ -8217,7 +8217,7 @@
           <t>ANGI-104</t>
         </is>
       </c>
-      <c r="M93" s="2" t="inlineStr"/>
+      <c r="M93" s="2"/>
       <c r="N93" s="2" t="n">
         <v>3.9</v>
       </c>
@@ -8292,7 +8292,7 @@
           <t>ANGI-105</t>
         </is>
       </c>
-      <c r="M94" s="2" t="inlineStr"/>
+      <c r="M94" s="2"/>
       <c r="N94" s="2" t="n">
         <v>8.5</v>
       </c>
@@ -8366,7 +8366,7 @@
           <t>ANGI-106</t>
         </is>
       </c>
-      <c r="M95" s="2" t="inlineStr"/>
+      <c r="M95" s="2"/>
       <c r="N95" s="2" t="n">
         <v>6</v>
       </c>
@@ -8439,7 +8439,7 @@
           <t>ANGI-107</t>
         </is>
       </c>
-      <c r="M96" s="2" t="inlineStr"/>
+      <c r="M96" s="2"/>
       <c r="N96" s="2" t="n">
         <v>6.1</v>
       </c>
@@ -8508,7 +8508,7 @@
           <t>ANGI-108</t>
         </is>
       </c>
-      <c r="M97" s="2" t="inlineStr"/>
+      <c r="M97" s="2"/>
       <c r="N97" s="2" t="n">
         <v>6.3</v>
       </c>
@@ -8581,7 +8581,7 @@
           <t>ANGI-109</t>
         </is>
       </c>
-      <c r="M98" s="2" t="inlineStr"/>
+      <c r="M98" s="2"/>
       <c r="N98" s="2" t="n">
         <v>6</v>
       </c>
@@ -8654,7 +8654,7 @@
           <t>ANGI-110</t>
         </is>
       </c>
-      <c r="M99" s="2" t="inlineStr"/>
+      <c r="M99" s="2"/>
       <c r="N99" s="2" t="n">
         <v>8</v>
       </c>
@@ -8728,7 +8728,7 @@
           <t>ANGI-111</t>
         </is>
       </c>
-      <c r="M100" s="2" t="inlineStr"/>
+      <c r="M100" s="2"/>
       <c r="N100" s="2" t="n">
         <v>5.6</v>
       </c>
@@ -8802,7 +8802,7 @@
           <t>ANGI-112</t>
         </is>
       </c>
-      <c r="M101" s="2" t="inlineStr"/>
+      <c r="M101" s="2"/>
       <c r="N101" s="2" t="n">
         <v>7.8</v>
       </c>
@@ -8871,7 +8871,7 @@
           <t>ANGI-113</t>
         </is>
       </c>
-      <c r="M102" s="2" t="inlineStr"/>
+      <c r="M102" s="2"/>
       <c r="N102" s="2" t="n">
         <v>46</v>
       </c>
@@ -8946,7 +8946,7 @@
           <t>ANGI-114</t>
         </is>
       </c>
-      <c r="M103" s="2" t="inlineStr"/>
+      <c r="M103" s="2"/>
       <c r="N103" s="2" t="n">
         <v>5.1</v>
       </c>
@@ -9021,7 +9021,7 @@
           <t>ANGI-115</t>
         </is>
       </c>
-      <c r="M104" s="2" t="inlineStr"/>
+      <c r="M104" s="2"/>
       <c r="N104" s="2" t="n">
         <v>7.1</v>
       </c>
@@ -9094,7 +9094,7 @@
           <t>ANGI-116</t>
         </is>
       </c>
-      <c r="M105" s="2" t="inlineStr"/>
+      <c r="M105" s="2"/>
       <c r="N105" s="2" t="n">
         <v>7.1</v>
       </c>
@@ -9167,7 +9167,7 @@
           <t>ANGI-117</t>
         </is>
       </c>
-      <c r="M106" s="2" t="inlineStr"/>
+      <c r="M106" s="2"/>
       <c r="N106" s="2" t="n">
         <v>5.1</v>
       </c>
@@ -9240,7 +9240,7 @@
           <t>ANGI-118</t>
         </is>
       </c>
-      <c r="M107" s="2" t="inlineStr"/>
+      <c r="M107" s="2"/>
       <c r="N107" s="2" t="n">
         <v>4.8</v>
       </c>
@@ -9313,7 +9313,7 @@
           <t>ANGI-119</t>
         </is>
       </c>
-      <c r="M108" s="2" t="inlineStr"/>
+      <c r="M108" s="2"/>
       <c r="N108" s="2" t="n">
         <v>6.8</v>
       </c>
@@ -9387,7 +9387,7 @@
           <t>ANGI-120</t>
         </is>
       </c>
-      <c r="M109" s="2" t="inlineStr"/>
+      <c r="M109" s="2"/>
       <c r="N109" s="2" t="n">
         <v>6.4</v>
       </c>
@@ -9460,7 +9460,7 @@
           <t>ANGI-121</t>
         </is>
       </c>
-      <c r="M110" s="2" t="inlineStr"/>
+      <c r="M110" s="2"/>
       <c r="N110" s="2" t="n">
         <v>4.6</v>
       </c>
@@ -9529,7 +9529,7 @@
           <t>ANGI-122</t>
         </is>
       </c>
-      <c r="M111" s="2" t="inlineStr"/>
+      <c r="M111" s="2"/>
       <c r="N111" s="2" t="n">
         <v>6.3</v>
       </c>
@@ -9602,7 +9602,7 @@
           <t>ANGI-123</t>
         </is>
       </c>
-      <c r="M112" s="2" t="inlineStr"/>
+      <c r="M112" s="2"/>
       <c r="N112" s="2" t="n">
         <v>4.4</v>
       </c>
@@ -9677,7 +9677,7 @@
           <t>ANGI-124</t>
         </is>
       </c>
-      <c r="M113" s="2" t="inlineStr"/>
+      <c r="M113" s="2"/>
       <c r="N113" s="2" t="n">
         <v>3.3</v>
       </c>
@@ -9751,7 +9751,7 @@
           <t>ANGI-125</t>
         </is>
       </c>
-      <c r="M114" s="2" t="inlineStr"/>
+      <c r="M114" s="2"/>
       <c r="N114" s="2" t="n">
         <v>5.9</v>
       </c>
@@ -9824,7 +9824,7 @@
           <t>ANGI-126</t>
         </is>
       </c>
-      <c r="M115" s="2" t="inlineStr"/>
+      <c r="M115" s="2"/>
       <c r="N115" s="2" t="n">
         <v>5.7</v>
       </c>
@@ -9900,7 +9900,7 @@
           <t>ANGI-127</t>
         </is>
       </c>
-      <c r="M116" s="2" t="inlineStr"/>
+      <c r="M116" s="2"/>
       <c r="N116" s="2" t="n">
         <v>3.9</v>
       </c>
@@ -9975,7 +9975,7 @@
           <t>ANGI-128</t>
         </is>
       </c>
-      <c r="M117" s="2" t="inlineStr"/>
+      <c r="M117" s="2"/>
       <c r="N117" s="2" t="n">
         <v>1.7</v>
       </c>
@@ -10049,7 +10049,7 @@
           <t>ANGI-129</t>
         </is>
       </c>
-      <c r="M118" s="2" t="inlineStr"/>
+      <c r="M118" s="2"/>
       <c r="N118" s="2" t="n">
         <v>3.3</v>
       </c>
@@ -10123,7 +10123,7 @@
           <t>ANGI-130</t>
         </is>
       </c>
-      <c r="M119" s="2" t="inlineStr"/>
+      <c r="M119" s="2"/>
       <c r="N119" s="2" t="n">
         <v>5.4</v>
       </c>
@@ -10197,7 +10197,7 @@
           <t>ANGI-131</t>
         </is>
       </c>
-      <c r="M120" s="2" t="inlineStr"/>
+      <c r="M120" s="2"/>
       <c r="N120" s="2" t="n">
         <v>3.2</v>
       </c>
@@ -10270,7 +10270,7 @@
           <t>ANGI-132</t>
         </is>
       </c>
-      <c r="M121" s="2" t="inlineStr"/>
+      <c r="M121" s="2"/>
       <c r="N121" s="2" t="n">
         <v>2.1</v>
       </c>
@@ -10343,7 +10343,7 @@
           <t>ANGI-133</t>
         </is>
       </c>
-      <c r="M122" s="2" t="inlineStr"/>
+      <c r="M122" s="2"/>
       <c r="N122" s="2" t="n">
         <v>4.8</v>
       </c>
@@ -10416,7 +10416,7 @@
           <t>ANGI-134</t>
         </is>
       </c>
-      <c r="M123" s="2" t="inlineStr"/>
+      <c r="M123" s="2"/>
       <c r="N123" s="2" t="n">
         <v>5</v>
       </c>
@@ -10489,7 +10489,7 @@
           <t>ANGI-135</t>
         </is>
       </c>
-      <c r="M124" s="2" t="inlineStr"/>
+      <c r="M124" s="2"/>
       <c r="N124" s="2" t="n">
         <v>2.7</v>
       </c>
@@ -10562,7 +10562,7 @@
           <t>ANGI-136</t>
         </is>
       </c>
-      <c r="M125" s="2" t="inlineStr"/>
+      <c r="M125" s="2"/>
       <c r="N125" s="2" t="n">
         <v>4.6</v>
       </c>
@@ -10716,7 +10716,7 @@
           <t>ANGI-138</t>
         </is>
       </c>
-      <c r="M127" s="2" t="inlineStr"/>
+      <c r="M127" s="2"/>
       <c r="N127" s="2" t="n">
         <v>3.3</v>
       </c>
@@ -10790,7 +10790,7 @@
           <t>ANGI-139</t>
         </is>
       </c>
-      <c r="M128" s="2" t="inlineStr"/>
+      <c r="M128" s="2"/>
       <c r="N128" s="2" t="n">
         <v>1.9</v>
       </c>
@@ -10866,7 +10866,7 @@
           <t>ANGI-140</t>
         </is>
       </c>
-      <c r="M129" s="2" t="inlineStr"/>
+      <c r="M129" s="2"/>
       <c r="N129" s="2" t="n">
         <v>3.9</v>
       </c>
@@ -11182,7 +11182,7 @@
           <t>ANGI-144</t>
         </is>
       </c>
-      <c r="M133" s="2" t="inlineStr"/>
+      <c r="M133" s="2"/>
       <c r="N133" s="2" t="n">
         <v>1.6</v>
       </c>
@@ -11256,7 +11256,7 @@
           <t>ANGI-145</t>
         </is>
       </c>
-      <c r="M134" s="2" t="inlineStr"/>
+      <c r="M134" s="2"/>
       <c r="N134" s="2" t="n">
         <v>3.2</v>
       </c>
@@ -11412,7 +11412,7 @@
           <t>ANGI-147</t>
         </is>
       </c>
-      <c r="M136" s="2" t="inlineStr"/>
+      <c r="M136" s="2"/>
       <c r="N136" s="2" t="n">
         <v>2.5</v>
       </c>
@@ -11485,7 +11485,7 @@
           <t>ANGI-148</t>
         </is>
       </c>
-      <c r="M137" s="2" t="inlineStr"/>
+      <c r="M137" s="2"/>
       <c r="N137" s="2" t="n">
         <v>2.8</v>
       </c>
@@ -11558,7 +11558,7 @@
           <t>ANGI-149</t>
         </is>
       </c>
-      <c r="M138" s="2" t="inlineStr"/>
+      <c r="M138" s="2"/>
       <c r="N138" s="2" t="n">
         <v>2.2</v>
       </c>
@@ -11631,7 +11631,7 @@
           <t>ANGI-150</t>
         </is>
       </c>
-      <c r="M139" s="2" t="inlineStr"/>
+      <c r="M139" s="2"/>
       <c r="N139" s="2" t="n">
         <v>2.1</v>
       </c>
@@ -11787,7 +11787,7 @@
           <t>ANGI-152</t>
         </is>
       </c>
-      <c r="M141" s="2" t="inlineStr"/>
+      <c r="M141" s="2"/>
       <c r="N141" s="2" t="n">
         <v>1.6</v>
       </c>
@@ -12020,7 +12020,7 @@
           <t>ANGI-155</t>
         </is>
       </c>
-      <c r="M144" s="2" t="inlineStr"/>
+      <c r="M144" s="2"/>
       <c r="N144" s="2" t="n">
         <v>40</v>
       </c>
@@ -12699,7 +12699,7 @@
           <t>ANGI-164</t>
         </is>
       </c>
-      <c r="M153" s="2" t="inlineStr"/>
+      <c r="M153" s="2"/>
       <c r="N153" s="2" t="n">
         <v>8</v>
       </c>
@@ -12768,7 +12768,7 @@
           <t>ANGI-165</t>
         </is>
       </c>
-      <c r="M154" s="2" t="inlineStr"/>
+      <c r="M154" s="2"/>
       <c r="N154" s="2" t="n">
         <v>36</v>
       </c>
@@ -12918,7 +12918,7 @@
           <t>ANGI-167</t>
         </is>
       </c>
-      <c r="M156" s="2" t="inlineStr"/>
+      <c r="M156" s="2"/>
       <c r="N156" s="2" t="n">
         <v>7.4</v>
       </c>
@@ -12992,7 +12992,7 @@
           <t>ANGI-168</t>
         </is>
       </c>
-      <c r="M157" s="2" t="inlineStr"/>
+      <c r="M157" s="2"/>
       <c r="N157" s="2" t="n">
         <v>8.6</v>
       </c>
@@ -13068,7 +13068,7 @@
           <t>ANGI-169</t>
         </is>
       </c>
-      <c r="M158" s="2" t="inlineStr"/>
+      <c r="M158" s="2"/>
       <c r="N158" s="2" t="n">
         <v>6.4</v>
       </c>
@@ -13145,7 +13145,7 @@
           <t>ANGI-170</t>
         </is>
       </c>
-      <c r="M159" s="2" t="inlineStr"/>
+      <c r="M159" s="2"/>
       <c r="N159" s="2" t="n">
         <v>4.7</v>
       </c>
@@ -13221,7 +13221,7 @@
           <t>ANGI-171</t>
         </is>
       </c>
-      <c r="M160" s="2" t="inlineStr"/>
+      <c r="M160" s="2"/>
       <c r="N160" s="2" t="n">
         <v>8.800000000000001</v>
       </c>
@@ -13290,7 +13290,7 @@
           <t>ANGI-172</t>
         </is>
       </c>
-      <c r="M161" s="2" t="inlineStr"/>
+      <c r="M161" s="2"/>
       <c r="N161" s="2" t="n">
         <v>4.9</v>
       </c>
@@ -13364,7 +13364,7 @@
           <t>ANGI-173</t>
         </is>
       </c>
-      <c r="M162" s="2" t="inlineStr"/>
+      <c r="M162" s="2"/>
       <c r="N162" s="2" t="n">
         <v>5.5</v>
       </c>
@@ -13440,7 +13440,7 @@
           <t>ANGI-174</t>
         </is>
       </c>
-      <c r="M163" s="2" t="inlineStr"/>
+      <c r="M163" s="2"/>
       <c r="N163" s="2" t="n">
         <v>7.2</v>
       </c>
@@ -13516,7 +13516,7 @@
           <t>ANGI-175</t>
         </is>
       </c>
-      <c r="M164" s="2" t="inlineStr"/>
+      <c r="M164" s="2"/>
       <c r="N164" s="2" t="n">
         <v>5.3</v>
       </c>
@@ -13592,7 +13592,7 @@
           <t>ANGI-176</t>
         </is>
       </c>
-      <c r="M165" s="2" t="inlineStr"/>
+      <c r="M165" s="2"/>
       <c r="N165" s="2" t="n">
         <v>7.7</v>
       </c>
@@ -13661,7 +13661,7 @@
           <t>ANGI-177</t>
         </is>
       </c>
-      <c r="M166" s="2" t="inlineStr"/>
+      <c r="M166" s="2"/>
       <c r="N166" s="2" t="n">
         <v>32</v>
       </c>
@@ -13736,7 +13736,7 @@
           <t>ANGI-178</t>
         </is>
       </c>
-      <c r="M167" s="2" t="inlineStr"/>
+      <c r="M167" s="2"/>
       <c r="N167" s="2" t="n">
         <v>4.3</v>
       </c>
@@ -13812,7 +13812,7 @@
           <t>ANGI-179</t>
         </is>
       </c>
-      <c r="M168" s="2" t="inlineStr"/>
+      <c r="M168" s="2"/>
       <c r="N168" s="2" t="n">
         <v>4.8</v>
       </c>
@@ -13886,7 +13886,7 @@
           <t>ANGI-180</t>
         </is>
       </c>
-      <c r="M169" s="2" t="inlineStr"/>
+      <c r="M169" s="2"/>
       <c r="N169" s="2" t="n">
         <v>5.8</v>
       </c>
@@ -13962,7 +13962,7 @@
           <t>ANGI-181</t>
         </is>
       </c>
-      <c r="M170" s="2" t="inlineStr"/>
+      <c r="M170" s="2"/>
       <c r="N170" s="2" t="n">
         <v>5.7</v>
       </c>
@@ -14035,7 +14035,7 @@
           <t>ANGI-182</t>
         </is>
       </c>
-      <c r="M171" s="2" t="inlineStr"/>
+      <c r="M171" s="2"/>
       <c r="N171" s="2" t="n">
         <v>4.5</v>
       </c>
@@ -14110,7 +14110,7 @@
           <t>ANGI-183</t>
         </is>
       </c>
-      <c r="M172" s="2" t="inlineStr"/>
+      <c r="M172" s="2"/>
       <c r="N172" s="2" t="n">
         <v>3.9</v>
       </c>
@@ -14187,7 +14187,7 @@
           <t>ANGI-184</t>
         </is>
       </c>
-      <c r="M173" s="2" t="inlineStr"/>
+      <c r="M173" s="2"/>
       <c r="N173" s="2" t="n">
         <v>2.7</v>
       </c>
@@ -14256,7 +14256,7 @@
           <t>ANGI-185</t>
         </is>
       </c>
-      <c r="M174" s="2" t="inlineStr"/>
+      <c r="M174" s="2"/>
       <c r="N174" s="2" t="n">
         <v>4.9</v>
       </c>
@@ -14329,7 +14329,7 @@
           <t>ANGI-186</t>
         </is>
       </c>
-      <c r="M175" s="2" t="inlineStr"/>
+      <c r="M175" s="2"/>
       <c r="N175" s="2" t="n">
         <v>3.2</v>
       </c>
@@ -14405,7 +14405,7 @@
           <t>ANGI-187</t>
         </is>
       </c>
-      <c r="M176" s="2" t="inlineStr"/>
+      <c r="M176" s="2"/>
       <c r="N176" s="2" t="n">
         <v>4.5</v>
       </c>
@@ -14479,7 +14479,7 @@
           <t>ANGI-188</t>
         </is>
       </c>
-      <c r="M177" s="2" t="inlineStr"/>
+      <c r="M177" s="2"/>
       <c r="N177" s="2" t="n">
         <v>4.9</v>
       </c>
@@ -14556,7 +14556,7 @@
           <t>ANGI-189</t>
         </is>
       </c>
-      <c r="M178" s="2" t="inlineStr"/>
+      <c r="M178" s="2"/>
       <c r="N178" s="2" t="n">
         <v>1.6</v>
       </c>
@@ -14629,7 +14629,7 @@
           <t>ANGI-190</t>
         </is>
       </c>
-      <c r="M179" s="2" t="inlineStr"/>
+      <c r="M179" s="2"/>
       <c r="N179" s="2" t="n">
         <v>3.8</v>
       </c>
@@ -14706,7 +14706,7 @@
           <t>ANGI-191</t>
         </is>
       </c>
-      <c r="M180" s="2" t="inlineStr"/>
+      <c r="M180" s="2"/>
       <c r="N180" s="2" t="n">
         <v>2</v>
       </c>
@@ -14781,7 +14781,7 @@
           <t>ANGI-192</t>
         </is>
       </c>
-      <c r="M181" s="2" t="inlineStr"/>
+      <c r="M181" s="2"/>
       <c r="N181" s="2" t="n">
         <v>3.7</v>
       </c>
@@ -14850,7 +14850,7 @@
           <t>ANGI-193</t>
         </is>
       </c>
-      <c r="M182" s="2" t="inlineStr"/>
+      <c r="M182" s="2"/>
       <c r="N182" s="2" t="n">
         <v>3</v>
       </c>
@@ -15090,7 +15090,7 @@
           <t>ANGI-196</t>
         </is>
       </c>
-      <c r="M185" s="2" t="inlineStr"/>
+      <c r="M185" s="2"/>
       <c r="N185" s="2" t="n">
         <v>2.6</v>
       </c>
@@ -15165,7 +15165,7 @@
           <t>ANGI-197</t>
         </is>
       </c>
-      <c r="M186" s="2" t="inlineStr"/>
+      <c r="M186" s="2"/>
       <c r="N186" s="2" t="n">
         <v>2.4</v>
       </c>
@@ -15324,7 +15324,7 @@
           <t>ANGI-199</t>
         </is>
       </c>
-      <c r="M188" s="2" t="inlineStr"/>
+      <c r="M188" s="2"/>
       <c r="N188" s="2" t="n">
         <v>1.8</v>
       </c>
@@ -15478,7 +15478,7 @@
           <t>ANGI-201</t>
         </is>
       </c>
-      <c r="M190" s="2" t="inlineStr"/>
+      <c r="M190" s="2"/>
       <c r="N190" s="2" t="n">
         <v>26</v>
       </c>
@@ -16772,7 +16772,7 @@
           <t>ANGI-218</t>
         </is>
       </c>
-      <c r="M207" s="2" t="inlineStr"/>
+      <c r="M207" s="2"/>
       <c r="N207" s="2" t="n">
         <v>12</v>
       </c>
@@ -16841,7 +16841,7 @@
           <t>ANGI-219</t>
         </is>
       </c>
-      <c r="M208" s="2" t="inlineStr"/>
+      <c r="M208" s="2"/>
       <c r="N208" s="2" t="n">
         <v>2</v>
       </c>
@@ -17158,8 +17158,67 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T231</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Task</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[BE] Implement Agent roadmap conversations MVP</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implement AGENT-01..04 from ANGI_Agent_Implementation_Ver1.1: expiring memory, leased/idempotent turns, scoped validated proposals, atomic create/update confirmation, roadmap revisions, cleanup and tests. API/Data Dictionary additions accompany source. Refs: ANGI-231.</t>
+        </is>
+      </c>
+      <c r="E213" s="2">
+      </c>
+      <c r="F213" s="2">
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EP-ROAD</t>
+        </is>
+      </c>
+      <c r="H213" s="2">
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26/10/2026</t>
+        </is>
+      </c>
+      <c r="J213" s="2">
+      </c>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend agent roadmap</t>
+        </is>
+      </c>
+      <c r="L213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANGI-231</t>
+        </is>
+      </c>
+      <c r="M213" s="2">
+      </c>
+      <c r="N213" s="2">
+      </c>
+      <c r="O213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O212"/>
+  <autoFilter ref="A1:O213"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17170,7 +17229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX212"/>
+  <dimension ref="A1:BX213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28513,6 +28572,71 @@
       <c r="BW212" s="9" t="n"/>
       <c r="BX212" s="9" t="n"/>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANGI-231</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[BE] Implement Agent roadmap conversations MVP</t>
+        </is>
+      </c>
+      <c r="C213">
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26/10/2026</t>
+        </is>
+      </c>
+      <c r="E213">
+      </c>
+      <c r="F213">
+      </c>
+      <c r="G213">
+      </c>
+      <c r="L213" s="7">
+      </c>
+      <c r="M213" s="7">
+      </c>
+      <c r="S213" s="7">
+      </c>
+      <c r="T213" s="7">
+      </c>
+      <c r="Z213" s="7">
+      </c>
+      <c r="AA213" s="7">
+      </c>
+      <c r="AG213" s="7">
+      </c>
+      <c r="AH213" s="7">
+      </c>
+      <c r="AN213" s="7">
+      </c>
+      <c r="AO213" s="7">
+      </c>
+      <c r="AU213" s="7">
+      </c>
+      <c r="AV213" s="7">
+      </c>
+      <c r="BB213" s="7">
+      </c>
+      <c r="BC213" s="7">
+      </c>
+      <c r="BI213" s="7">
+      </c>
+      <c r="BJ213" s="7">
+      </c>
+      <c r="BP213" s="7">
+      </c>
+      <c r="BQ213" s="7">
+      </c>
+      <c r="BW213" s="7">
+      </c>
+      <c r="BX213" s="7">
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28524,7 +28648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -28719,7 +28843,8 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7"/>
+    <row r="7">
+    </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>

</xml_diff>